<commit_message>
chore(dr): bump settle-dr-dune to 903f844 — June 2026 DR lands
Update the settle-dr-dune submodule 2a4e204 → 903f844 (their PR #7:
queries ported to openmsc, DR settled through June 2026) and refresh
Distribution Rewards via `--dr-only` (no recompute).

June DR fills the known TBD gap for all four DR primes:
  Spark 1,650,764.59 · Skybase 164,694.33 · Grove 55,456.33 ·
  Keel 19,571.76 — June prime profits rise by the same.

Jan–May totals unchanged. The openmsc port adds three zero-value ref
codes (100/184/999) to Spark's table and swaps the labels of the
untagged spUSDT/spUSDC synthetic codes (130 ↔ 131; values exchanged,
sums identical). Grove gains ref code 2013 (zero through May).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
+++ b/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -505,168 +505,178 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" s="4" t="n">
-        <v>2960358.323387762</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>+ distribution_rewards (settle-dr-dune)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>55456.33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" s="4" t="n">
+        <v>3015814.653387762</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>3291039.781244973</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>3291039.781244973</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B11" s="3" t="n">
         <v>4709026.177726324</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" s="4" t="n">
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" s="4" t="n">
         <v>8000065.958971297</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Sky Revenue (max) — BR × full ilk debt, no deductions</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CoF on Net_Subs (actual BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>3291039.781244973</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>CoF on Net_Subs (actual BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>3291039.781244973</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>reduction from idle/SDE deductions</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B16" s="3" t="n">
         <v>-4934411.090697014</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" s="4" t="n">
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" s="4" t="n">
         <v>8225450.871941987</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>2893733.700012341</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>2893733.700012341</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B21" s="3" t="n">
         <v>-3291039.781244973</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" s="4" t="n">
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" s="4" t="n">
         <v>-397306.081232632</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-06-01 → 2026-06-30 (30 days)</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>avalanche_c=89166730, base=48037326, ethereum=25433938, monad=84784216, plume=78267500</t>
+          <t>2026-06-01 → 2026-06-30 (30 days)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-03T06:36:22+00:00</t>
+          <t>avalanche_c=89166730, base=48037326, ethereum=25433938, monad=84784216, plume=78267500</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-07T14:51:44+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>

<commit_message>
chore(dr): bump settle-dr-dune to 903f844 — June 2026 DR lands (#145)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
+++ b/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -505,168 +505,178 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" s="4" t="n">
-        <v>2960358.323387762</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>+ distribution_rewards (settle-dr-dune)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>55456.33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" s="4" t="n">
+        <v>3015814.653387762</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>3291039.781244973</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>3291039.781244973</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B11" s="3" t="n">
         <v>4709026.177726324</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" s="4" t="n">
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" s="4" t="n">
         <v>8000065.958971297</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Sky Revenue (max) — BR × full ilk debt, no deductions</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CoF on Net_Subs (actual BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>3291039.781244973</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>CoF on Net_Subs (actual BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>3291039.781244973</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>reduction from idle/SDE deductions</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B16" s="3" t="n">
         <v>-4934411.090697014</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" s="4" t="n">
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" s="4" t="n">
         <v>8225450.871941987</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>2893733.700012341</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>2893733.700012341</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B21" s="3" t="n">
         <v>-3291039.781244973</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" s="4" t="n">
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" s="4" t="n">
         <v>-397306.081232632</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-06-01 → 2026-06-30 (30 days)</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>avalanche_c=89166730, base=48037326, ethereum=25433938, monad=84784216, plume=78267500</t>
+          <t>2026-06-01 → 2026-06-30 (30 days)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-03T06:36:22+00:00</t>
+          <t>avalanche_c=89166730, base=48037326, ethereum=25433938, monad=84784216, plume=78267500</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-07T14:51:44+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): regenerate spark under recovered aToken yield
March: S9 +$162,936.93 (mid-month entry), S2 +$32,005.46 (staged exit) —
supply-side 2,350,300.04 → 2,545,242.43. April: S9 +$467,640.35 (exit
month), S54 +$4,618.66 — supply-side 834,856.97 → 1,307,115.98. Remaining
months carry only 1-raw-unit ROUND_HALF_EVEN harmonization.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
+++ b/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-10T11:17:39+00:00</t>
+          <t>2026-07-13T18:40:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1958,13 +1958,13 @@
         <v>0.000702235016912599</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.000702235016912598</v>
+        <v>0.000702235016912599</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.000702235016912598</v>
+        <v>0.000702235016912599</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
@@ -1982,7 +1982,7 @@
         <v>0.001110606709394735</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-0.0004083716924821368</v>
+        <v>-0.0004083716924821358</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(spark): recover Cat C aToken yield for mid-window entry/exit (S9/S2/S54) (#149)
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
+++ b/settlements/grove/2026-06/grove_settlement_june_2026.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-10T11:17:39+00:00</t>
+          <t>2026-07-13T18:40:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1958,13 +1958,13 @@
         <v>0.000702235016912599</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.000702235016912598</v>
+        <v>0.000702235016912599</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.000702235016912598</v>
+        <v>0.000702235016912599</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
@@ -1982,7 +1982,7 @@
         <v>0.001110606709394735</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-0.0004083716924821368</v>
+        <v>-0.0004083716924821358</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>

</xml_diff>